<commit_message>
Sayt tuzatishlari: aniq xatolar, tez rasmlar, kunni yopish soati; Code.gs yangilandi
</commit_message>
<xml_diff>
--- a/SmartSchool_Sheets_shablon.xlsx
+++ b/SmartSchool_Sheets_shablon.xlsx
@@ -12,6 +12,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Attendance" sheetId="3" state="visible" r:id="rId3"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Events" sheetId="4" state="visible" r:id="rId4"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Audit" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Settings" sheetId="6" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -21,7 +22,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="7">
+  <fonts count="10">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -59,6 +60,18 @@
       <name val="Arial"/>
       <b val="1"/>
       <sz val="10"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
     </font>
   </fonts>
   <fills count="4">
@@ -105,7 +118,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="12">
+  <cellXfs count="16">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -134,6 +147,12 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="49" fontId="8" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -499,7 +518,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F51"/>
+  <dimension ref="A1:F53"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -520,7 +539,7 @@
     <row r="3" ht="32" customHeight="1">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>1. Google Sheets da yangi jadval oching (sheets.new). Pastdagi 4 ta varaq nomi AYNAN shunday bo'lsin: Students, Attendance, Events, Audit.</t>
+          <t>1. Google Sheets da yangi jadval oching (sheets.new). Pastdagi 5 ta varaq nomi AYNAN shunday bo'lsin: Students, Attendance, Events, Audit, Settings.</t>
         </is>
       </c>
     </row>
@@ -1647,6 +1666,13 @@
       <c r="F51" s="8" t="inlineStr">
         <is>
           <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="12" t="inlineStr">
+        <is>
+          <t>Settings varag'i: SCHOOL, START, END, TZ, MINGAP — sozlamalar (saytdan o'zgaradi, Python ham o'qiydi). HB_* qatorlarini Python o'zi yozadi (kamera holati). Bu qiymatlar namuna emas, haqiqiy boshlang'ich sozlamalar.</t>
         </is>
       </c>
     </row>
@@ -25908,4 +25934,705 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:B200"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="16" customWidth="1" min="1" max="1"/>
+    <col width="22" customWidth="1" min="2" max="2"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="13" t="inlineStr">
+        <is>
+          <t>key</t>
+        </is>
+      </c>
+      <c r="B1" s="13" t="inlineStr">
+        <is>
+          <t>value</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="14" t="inlineStr">
+        <is>
+          <t>SCHOOL</t>
+        </is>
+      </c>
+      <c r="B2" s="15" t="inlineStr">
+        <is>
+          <t>Maktab</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="14" t="inlineStr">
+        <is>
+          <t>START</t>
+        </is>
+      </c>
+      <c r="B3" s="15" t="inlineStr">
+        <is>
+          <t>08:30</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="14" t="inlineStr">
+        <is>
+          <t>END</t>
+        </is>
+      </c>
+      <c r="B4" s="15" t="inlineStr">
+        <is>
+          <t>13:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="14" t="inlineStr">
+        <is>
+          <t>TZ</t>
+        </is>
+      </c>
+      <c r="B5" s="15" t="inlineStr">
+        <is>
+          <t>Asia/Tashkent</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="14" t="inlineStr">
+        <is>
+          <t>MINGAP</t>
+        </is>
+      </c>
+      <c r="B6" s="15" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="14" t="inlineStr">
+        <is>
+          <t>CLOSE_HOUR</t>
+        </is>
+      </c>
+      <c r="B7" s="15" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="14" t="inlineStr">
+        <is>
+          <t>HB_T</t>
+        </is>
+      </c>
+      <c r="B8" s="15" t="inlineStr"/>
+    </row>
+    <row r="9">
+      <c r="A9" s="14" t="inlineStr">
+        <is>
+          <t>HB_FPS</t>
+        </is>
+      </c>
+      <c r="B9" s="15" t="inlineStr"/>
+    </row>
+    <row r="10">
+      <c r="A10" s="14" t="inlineStr">
+        <is>
+          <t>HB_CAM</t>
+        </is>
+      </c>
+      <c r="B10" s="15" t="inlineStr"/>
+    </row>
+    <row r="11">
+      <c r="A11" s="14" t="inlineStr">
+        <is>
+          <t>HB_HOST</t>
+        </is>
+      </c>
+      <c r="B11" s="15" t="inlineStr"/>
+    </row>
+    <row r="12">
+      <c r="B12" s="11" t="n"/>
+    </row>
+    <row r="13">
+      <c r="B13" s="11" t="n"/>
+    </row>
+    <row r="14">
+      <c r="B14" s="11" t="n"/>
+    </row>
+    <row r="15">
+      <c r="B15" s="11" t="n"/>
+    </row>
+    <row r="16">
+      <c r="B16" s="11" t="n"/>
+    </row>
+    <row r="17">
+      <c r="B17" s="11" t="n"/>
+    </row>
+    <row r="18">
+      <c r="B18" s="11" t="n"/>
+    </row>
+    <row r="19">
+      <c r="B19" s="11" t="n"/>
+    </row>
+    <row r="20">
+      <c r="B20" s="11" t="n"/>
+    </row>
+    <row r="21">
+      <c r="B21" s="11" t="n"/>
+    </row>
+    <row r="22">
+      <c r="B22" s="11" t="n"/>
+    </row>
+    <row r="23">
+      <c r="B23" s="11" t="n"/>
+    </row>
+    <row r="24">
+      <c r="B24" s="11" t="n"/>
+    </row>
+    <row r="25">
+      <c r="B25" s="11" t="n"/>
+    </row>
+    <row r="26">
+      <c r="B26" s="11" t="n"/>
+    </row>
+    <row r="27">
+      <c r="B27" s="11" t="n"/>
+    </row>
+    <row r="28">
+      <c r="B28" s="11" t="n"/>
+    </row>
+    <row r="29">
+      <c r="B29" s="11" t="n"/>
+    </row>
+    <row r="30">
+      <c r="B30" s="11" t="n"/>
+    </row>
+    <row r="31">
+      <c r="B31" s="11" t="n"/>
+    </row>
+    <row r="32">
+      <c r="B32" s="11" t="n"/>
+    </row>
+    <row r="33">
+      <c r="B33" s="11" t="n"/>
+    </row>
+    <row r="34">
+      <c r="B34" s="11" t="n"/>
+    </row>
+    <row r="35">
+      <c r="B35" s="11" t="n"/>
+    </row>
+    <row r="36">
+      <c r="B36" s="11" t="n"/>
+    </row>
+    <row r="37">
+      <c r="B37" s="11" t="n"/>
+    </row>
+    <row r="38">
+      <c r="B38" s="11" t="n"/>
+    </row>
+    <row r="39">
+      <c r="B39" s="11" t="n"/>
+    </row>
+    <row r="40">
+      <c r="B40" s="11" t="n"/>
+    </row>
+    <row r="41">
+      <c r="B41" s="11" t="n"/>
+    </row>
+    <row r="42">
+      <c r="B42" s="11" t="n"/>
+    </row>
+    <row r="43">
+      <c r="B43" s="11" t="n"/>
+    </row>
+    <row r="44">
+      <c r="B44" s="11" t="n"/>
+    </row>
+    <row r="45">
+      <c r="B45" s="11" t="n"/>
+    </row>
+    <row r="46">
+      <c r="B46" s="11" t="n"/>
+    </row>
+    <row r="47">
+      <c r="B47" s="11" t="n"/>
+    </row>
+    <row r="48">
+      <c r="B48" s="11" t="n"/>
+    </row>
+    <row r="49">
+      <c r="B49" s="11" t="n"/>
+    </row>
+    <row r="50">
+      <c r="B50" s="11" t="n"/>
+    </row>
+    <row r="51">
+      <c r="B51" s="11" t="n"/>
+    </row>
+    <row r="52">
+      <c r="B52" s="11" t="n"/>
+    </row>
+    <row r="53">
+      <c r="B53" s="11" t="n"/>
+    </row>
+    <row r="54">
+      <c r="B54" s="11" t="n"/>
+    </row>
+    <row r="55">
+      <c r="B55" s="11" t="n"/>
+    </row>
+    <row r="56">
+      <c r="B56" s="11" t="n"/>
+    </row>
+    <row r="57">
+      <c r="B57" s="11" t="n"/>
+    </row>
+    <row r="58">
+      <c r="B58" s="11" t="n"/>
+    </row>
+    <row r="59">
+      <c r="B59" s="11" t="n"/>
+    </row>
+    <row r="60">
+      <c r="B60" s="11" t="n"/>
+    </row>
+    <row r="61">
+      <c r="B61" s="11" t="n"/>
+    </row>
+    <row r="62">
+      <c r="B62" s="11" t="n"/>
+    </row>
+    <row r="63">
+      <c r="B63" s="11" t="n"/>
+    </row>
+    <row r="64">
+      <c r="B64" s="11" t="n"/>
+    </row>
+    <row r="65">
+      <c r="B65" s="11" t="n"/>
+    </row>
+    <row r="66">
+      <c r="B66" s="11" t="n"/>
+    </row>
+    <row r="67">
+      <c r="B67" s="11" t="n"/>
+    </row>
+    <row r="68">
+      <c r="B68" s="11" t="n"/>
+    </row>
+    <row r="69">
+      <c r="B69" s="11" t="n"/>
+    </row>
+    <row r="70">
+      <c r="B70" s="11" t="n"/>
+    </row>
+    <row r="71">
+      <c r="B71" s="11" t="n"/>
+    </row>
+    <row r="72">
+      <c r="B72" s="11" t="n"/>
+    </row>
+    <row r="73">
+      <c r="B73" s="11" t="n"/>
+    </row>
+    <row r="74">
+      <c r="B74" s="11" t="n"/>
+    </row>
+    <row r="75">
+      <c r="B75" s="11" t="n"/>
+    </row>
+    <row r="76">
+      <c r="B76" s="11" t="n"/>
+    </row>
+    <row r="77">
+      <c r="B77" s="11" t="n"/>
+    </row>
+    <row r="78">
+      <c r="B78" s="11" t="n"/>
+    </row>
+    <row r="79">
+      <c r="B79" s="11" t="n"/>
+    </row>
+    <row r="80">
+      <c r="B80" s="11" t="n"/>
+    </row>
+    <row r="81">
+      <c r="B81" s="11" t="n"/>
+    </row>
+    <row r="82">
+      <c r="B82" s="11" t="n"/>
+    </row>
+    <row r="83">
+      <c r="B83" s="11" t="n"/>
+    </row>
+    <row r="84">
+      <c r="B84" s="11" t="n"/>
+    </row>
+    <row r="85">
+      <c r="B85" s="11" t="n"/>
+    </row>
+    <row r="86">
+      <c r="B86" s="11" t="n"/>
+    </row>
+    <row r="87">
+      <c r="B87" s="11" t="n"/>
+    </row>
+    <row r="88">
+      <c r="B88" s="11" t="n"/>
+    </row>
+    <row r="89">
+      <c r="B89" s="11" t="n"/>
+    </row>
+    <row r="90">
+      <c r="B90" s="11" t="n"/>
+    </row>
+    <row r="91">
+      <c r="B91" s="11" t="n"/>
+    </row>
+    <row r="92">
+      <c r="B92" s="11" t="n"/>
+    </row>
+    <row r="93">
+      <c r="B93" s="11" t="n"/>
+    </row>
+    <row r="94">
+      <c r="B94" s="11" t="n"/>
+    </row>
+    <row r="95">
+      <c r="B95" s="11" t="n"/>
+    </row>
+    <row r="96">
+      <c r="B96" s="11" t="n"/>
+    </row>
+    <row r="97">
+      <c r="B97" s="11" t="n"/>
+    </row>
+    <row r="98">
+      <c r="B98" s="11" t="n"/>
+    </row>
+    <row r="99">
+      <c r="B99" s="11" t="n"/>
+    </row>
+    <row r="100">
+      <c r="B100" s="11" t="n"/>
+    </row>
+    <row r="101">
+      <c r="B101" s="11" t="n"/>
+    </row>
+    <row r="102">
+      <c r="B102" s="11" t="n"/>
+    </row>
+    <row r="103">
+      <c r="B103" s="11" t="n"/>
+    </row>
+    <row r="104">
+      <c r="B104" s="11" t="n"/>
+    </row>
+    <row r="105">
+      <c r="B105" s="11" t="n"/>
+    </row>
+    <row r="106">
+      <c r="B106" s="11" t="n"/>
+    </row>
+    <row r="107">
+      <c r="B107" s="11" t="n"/>
+    </row>
+    <row r="108">
+      <c r="B108" s="11" t="n"/>
+    </row>
+    <row r="109">
+      <c r="B109" s="11" t="n"/>
+    </row>
+    <row r="110">
+      <c r="B110" s="11" t="n"/>
+    </row>
+    <row r="111">
+      <c r="B111" s="11" t="n"/>
+    </row>
+    <row r="112">
+      <c r="B112" s="11" t="n"/>
+    </row>
+    <row r="113">
+      <c r="B113" s="11" t="n"/>
+    </row>
+    <row r="114">
+      <c r="B114" s="11" t="n"/>
+    </row>
+    <row r="115">
+      <c r="B115" s="11" t="n"/>
+    </row>
+    <row r="116">
+      <c r="B116" s="11" t="n"/>
+    </row>
+    <row r="117">
+      <c r="B117" s="11" t="n"/>
+    </row>
+    <row r="118">
+      <c r="B118" s="11" t="n"/>
+    </row>
+    <row r="119">
+      <c r="B119" s="11" t="n"/>
+    </row>
+    <row r="120">
+      <c r="B120" s="11" t="n"/>
+    </row>
+    <row r="121">
+      <c r="B121" s="11" t="n"/>
+    </row>
+    <row r="122">
+      <c r="B122" s="11" t="n"/>
+    </row>
+    <row r="123">
+      <c r="B123" s="11" t="n"/>
+    </row>
+    <row r="124">
+      <c r="B124" s="11" t="n"/>
+    </row>
+    <row r="125">
+      <c r="B125" s="11" t="n"/>
+    </row>
+    <row r="126">
+      <c r="B126" s="11" t="n"/>
+    </row>
+    <row r="127">
+      <c r="B127" s="11" t="n"/>
+    </row>
+    <row r="128">
+      <c r="B128" s="11" t="n"/>
+    </row>
+    <row r="129">
+      <c r="B129" s="11" t="n"/>
+    </row>
+    <row r="130">
+      <c r="B130" s="11" t="n"/>
+    </row>
+    <row r="131">
+      <c r="B131" s="11" t="n"/>
+    </row>
+    <row r="132">
+      <c r="B132" s="11" t="n"/>
+    </row>
+    <row r="133">
+      <c r="B133" s="11" t="n"/>
+    </row>
+    <row r="134">
+      <c r="B134" s="11" t="n"/>
+    </row>
+    <row r="135">
+      <c r="B135" s="11" t="n"/>
+    </row>
+    <row r="136">
+      <c r="B136" s="11" t="n"/>
+    </row>
+    <row r="137">
+      <c r="B137" s="11" t="n"/>
+    </row>
+    <row r="138">
+      <c r="B138" s="11" t="n"/>
+    </row>
+    <row r="139">
+      <c r="B139" s="11" t="n"/>
+    </row>
+    <row r="140">
+      <c r="B140" s="11" t="n"/>
+    </row>
+    <row r="141">
+      <c r="B141" s="11" t="n"/>
+    </row>
+    <row r="142">
+      <c r="B142" s="11" t="n"/>
+    </row>
+    <row r="143">
+      <c r="B143" s="11" t="n"/>
+    </row>
+    <row r="144">
+      <c r="B144" s="11" t="n"/>
+    </row>
+    <row r="145">
+      <c r="B145" s="11" t="n"/>
+    </row>
+    <row r="146">
+      <c r="B146" s="11" t="n"/>
+    </row>
+    <row r="147">
+      <c r="B147" s="11" t="n"/>
+    </row>
+    <row r="148">
+      <c r="B148" s="11" t="n"/>
+    </row>
+    <row r="149">
+      <c r="B149" s="11" t="n"/>
+    </row>
+    <row r="150">
+      <c r="B150" s="11" t="n"/>
+    </row>
+    <row r="151">
+      <c r="B151" s="11" t="n"/>
+    </row>
+    <row r="152">
+      <c r="B152" s="11" t="n"/>
+    </row>
+    <row r="153">
+      <c r="B153" s="11" t="n"/>
+    </row>
+    <row r="154">
+      <c r="B154" s="11" t="n"/>
+    </row>
+    <row r="155">
+      <c r="B155" s="11" t="n"/>
+    </row>
+    <row r="156">
+      <c r="B156" s="11" t="n"/>
+    </row>
+    <row r="157">
+      <c r="B157" s="11" t="n"/>
+    </row>
+    <row r="158">
+      <c r="B158" s="11" t="n"/>
+    </row>
+    <row r="159">
+      <c r="B159" s="11" t="n"/>
+    </row>
+    <row r="160">
+      <c r="B160" s="11" t="n"/>
+    </row>
+    <row r="161">
+      <c r="B161" s="11" t="n"/>
+    </row>
+    <row r="162">
+      <c r="B162" s="11" t="n"/>
+    </row>
+    <row r="163">
+      <c r="B163" s="11" t="n"/>
+    </row>
+    <row r="164">
+      <c r="B164" s="11" t="n"/>
+    </row>
+    <row r="165">
+      <c r="B165" s="11" t="n"/>
+    </row>
+    <row r="166">
+      <c r="B166" s="11" t="n"/>
+    </row>
+    <row r="167">
+      <c r="B167" s="11" t="n"/>
+    </row>
+    <row r="168">
+      <c r="B168" s="11" t="n"/>
+    </row>
+    <row r="169">
+      <c r="B169" s="11" t="n"/>
+    </row>
+    <row r="170">
+      <c r="B170" s="11" t="n"/>
+    </row>
+    <row r="171">
+      <c r="B171" s="11" t="n"/>
+    </row>
+    <row r="172">
+      <c r="B172" s="11" t="n"/>
+    </row>
+    <row r="173">
+      <c r="B173" s="11" t="n"/>
+    </row>
+    <row r="174">
+      <c r="B174" s="11" t="n"/>
+    </row>
+    <row r="175">
+      <c r="B175" s="11" t="n"/>
+    </row>
+    <row r="176">
+      <c r="B176" s="11" t="n"/>
+    </row>
+    <row r="177">
+      <c r="B177" s="11" t="n"/>
+    </row>
+    <row r="178">
+      <c r="B178" s="11" t="n"/>
+    </row>
+    <row r="179">
+      <c r="B179" s="11" t="n"/>
+    </row>
+    <row r="180">
+      <c r="B180" s="11" t="n"/>
+    </row>
+    <row r="181">
+      <c r="B181" s="11" t="n"/>
+    </row>
+    <row r="182">
+      <c r="B182" s="11" t="n"/>
+    </row>
+    <row r="183">
+      <c r="B183" s="11" t="n"/>
+    </row>
+    <row r="184">
+      <c r="B184" s="11" t="n"/>
+    </row>
+    <row r="185">
+      <c r="B185" s="11" t="n"/>
+    </row>
+    <row r="186">
+      <c r="B186" s="11" t="n"/>
+    </row>
+    <row r="187">
+      <c r="B187" s="11" t="n"/>
+    </row>
+    <row r="188">
+      <c r="B188" s="11" t="n"/>
+    </row>
+    <row r="189">
+      <c r="B189" s="11" t="n"/>
+    </row>
+    <row r="190">
+      <c r="B190" s="11" t="n"/>
+    </row>
+    <row r="191">
+      <c r="B191" s="11" t="n"/>
+    </row>
+    <row r="192">
+      <c r="B192" s="11" t="n"/>
+    </row>
+    <row r="193">
+      <c r="B193" s="11" t="n"/>
+    </row>
+    <row r="194">
+      <c r="B194" s="11" t="n"/>
+    </row>
+    <row r="195">
+      <c r="B195" s="11" t="n"/>
+    </row>
+    <row r="196">
+      <c r="B196" s="11" t="n"/>
+    </row>
+    <row r="197">
+      <c r="B197" s="11" t="n"/>
+    </row>
+    <row r="198">
+      <c r="B198" s="11" t="n"/>
+    </row>
+    <row r="199">
+      <c r="B199" s="11" t="n"/>
+    </row>
+    <row r="200">
+      <c r="B200" s="11" t="n"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>